<commit_message>
Add completion % to SPECIALTY section in DASHBOARD
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="82">
+  <fonts count="83">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -571,6 +571,12 @@
       <name val="Arial"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="42">
     <fill>
@@ -947,7 +953,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="76" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1305,6 +1311,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="82" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -28887,7 +28899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="3" customWidth="1" style="104" min="1" max="1"/>
@@ -29310,7 +29322,32 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="4.2" customHeight="1" s="104"/>
+    <row r="36" ht="4.2" customHeight="1" s="104">
+      <c r="B36" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed")/C35,0)</f>
+        <v/>
+      </c>
+      <c r="C36" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C35,"0")</f>
+        <v/>
+      </c>
+      <c r="E36" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed")/F35,0)</f>
+        <v/>
+      </c>
+      <c r="F36" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F35,"0")</f>
+        <v/>
+      </c>
+      <c r="H36" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed")/I35,0)</f>
+        <v/>
+      </c>
+      <c r="I36" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I35,"0")</f>
+        <v/>
+      </c>
+    </row>
     <row r="37" ht="32.1" customHeight="1" s="104">
       <c r="B37" s="43" t="inlineStr">
         <is>
@@ -29340,7 +29377,32 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="4.2" customHeight="1" s="104"/>
+    <row r="38" ht="4.2" customHeight="1" s="104">
+      <c r="B38" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed")/C37,0)</f>
+        <v/>
+      </c>
+      <c r="C38" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C37,"0")</f>
+        <v/>
+      </c>
+      <c r="E38" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed")/F37,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F37,"0")</f>
+        <v/>
+      </c>
+      <c r="H38" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed")/I37,0)</f>
+        <v/>
+      </c>
+      <c r="I38" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I37,"0")</f>
+        <v/>
+      </c>
+    </row>
     <row r="39" ht="32.1" customHeight="1" s="104">
       <c r="B39" s="55" t="inlineStr">
         <is>
@@ -29370,7 +29432,32 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="4.2" customHeight="1" s="104"/>
+    <row r="40" ht="4.2" customHeight="1" s="104">
+      <c r="B40" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed")/C39,0)</f>
+        <v/>
+      </c>
+      <c r="C40" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C39,"0")</f>
+        <v/>
+      </c>
+      <c r="E40" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed")/F39,0)</f>
+        <v/>
+      </c>
+      <c r="F40" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F39,"0")</f>
+        <v/>
+      </c>
+      <c r="H40" s="125">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed")/I39,0)</f>
+        <v/>
+      </c>
+      <c r="I40" s="126">
+        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I39,"0")</f>
+        <v/>
+      </c>
+    </row>
     <row r="41" ht="32.1" customHeight="1" s="104"/>
   </sheetData>
   <mergeCells count="18">

</xml_diff>

<commit_message>
Fix specialty completion rows — expand hidden rows + correct formulas
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -574,11 +574,11 @@
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="00666666"/>
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -795,6 +795,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -953,7 +958,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="76" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1313,10 +1318,7 @@
     <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="82" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="82" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="82" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -29322,29 +29324,17 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="4.2" customHeight="1" s="104">
-      <c r="B36" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed")/C35,0)</f>
+    <row r="36" ht="14" customHeight="1" s="104">
+      <c r="C36" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="C36" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C35,"0")</f>
+      <c r="F36" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="E36" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed")/F35,0)</f>
-        <v/>
-      </c>
-      <c r="F36" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F35,"0")</f>
-        <v/>
-      </c>
-      <c r="H36" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed")/I35,0)</f>
-        <v/>
-      </c>
-      <c r="I36" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I35,"0")</f>
+      <c r="I36" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
     </row>
@@ -29377,29 +29367,17 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="4.2" customHeight="1" s="104">
-      <c r="B38" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed")/C37,0)</f>
+    <row r="38" ht="14" customHeight="1" s="104">
+      <c r="C38" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="C38" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C37,"0")</f>
+      <c r="F38" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="E38" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed")/F37,0)</f>
-        <v/>
-      </c>
-      <c r="F38" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F37,"0")</f>
-        <v/>
-      </c>
-      <c r="H38" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed")/I37,0)</f>
-        <v/>
-      </c>
-      <c r="I38" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I37,"0")</f>
+      <c r="I38" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
     </row>
@@ -29432,29 +29410,17 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="4.2" customHeight="1" s="104">
-      <c r="B40" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed")/C39,0)</f>
+    <row r="40" ht="14" customHeight="1" s="104">
+      <c r="C40" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="C40" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(C39,"0")</f>
+      <c r="F40" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
-      <c r="E40" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed")/F39,0)</f>
-        <v/>
-      </c>
-      <c r="F40" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(F39,"0")</f>
-        <v/>
-      </c>
-      <c r="H40" s="125">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed")/I39,0)</f>
-        <v/>
-      </c>
-      <c r="I40" s="126">
-        <f>TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(I39,"0")</f>
+      <c r="I40" s="125">
+        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP"),0),"0%")&amp;")","-")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix specialty completion — exact same formula pattern as Category
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="83">
+  <fonts count="84">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -577,6 +577,12 @@
       <color rgb="00666666"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF555555"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="43">
     <fill>
@@ -958,7 +964,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="76" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1319,6 +1325,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="82" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -29324,17 +29336,29 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="14" customHeight="1" s="104">
-      <c r="C36" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB"),0),"0%")&amp;")","-")</f>
+    <row r="36" ht="14.4" customHeight="1" s="104">
+      <c r="B36" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F36" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT"),0),"0%")&amp;")","-")</f>
+      <c r="C36" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"-")</f>
         <v/>
       </c>
-      <c r="I36" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV"),0),"0%")&amp;")","-")</f>
+      <c r="E36" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="F36" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"-")</f>
+        <v/>
+      </c>
+      <c r="H36" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="I36" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"-")</f>
         <v/>
       </c>
     </row>
@@ -29367,17 +29391,29 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="14" customHeight="1" s="104">
-      <c r="C38" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W"),0),"0%")&amp;")","-")</f>
+    <row r="38" ht="14.4" customHeight="1" s="104">
+      <c r="B38" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F38" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M"),0),"0%")&amp;")","-")</f>
+      <c r="C38" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"-")</f>
         <v/>
       </c>
-      <c r="I38" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT"),0),"0%")&amp;")","-")</f>
+      <c r="E38" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="F38" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"-")</f>
+        <v/>
+      </c>
+      <c r="H38" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="I38" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"-")</f>
         <v/>
       </c>
     </row>
@@ -29410,17 +29446,29 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="14" customHeight="1" s="104">
-      <c r="C40" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT"),0),"0%")&amp;")","-")</f>
+    <row r="40" ht="14.4" customHeight="1" s="104">
+      <c r="B40" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F40" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP"),0),"0%")&amp;")","-")</f>
+      <c r="C40" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"-")</f>
         <v/>
       </c>
-      <c r="I40" s="125">
-        <f>IFERROR(TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed"),"0")&amp;" / "&amp;TEXT(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP"),"0")&amp;"  ("&amp;TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP",'ASF Tracker'!E4:E1002,"Closed")/COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP"),0),"0%")&amp;")","-")</f>
+      <c r="E40" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="F40" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"-")</f>
+        <v/>
+      </c>
+      <c r="H40" s="126">
+        <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"0%"),"-")</f>
+        <v/>
+      </c>
+      <c r="I40" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"-")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Specialty: Closed/Total in count cell + Completion% row — matching Category style
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="84">
+  <fonts count="91">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -578,13 +578,53 @@
       <sz val="8"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="FF555555"/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF1565C0"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF6A1B9A"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF37474F"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF2E7D32"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF4E342E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFB71C1C"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFE65100"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="43">
+  <fills count="50">
     <fill>
       <patternFill/>
     </fill>
@@ -806,6 +846,41 @@
         <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEADAF5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE0E6EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD7EED9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE4DCD9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD8DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD9AD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -964,7 +1039,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="76" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="142">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="56" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1327,10 +1402,52 @@
     <xf numFmtId="0" fontId="82" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="83" fillId="23" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="83" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="85" fillId="24" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="25" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="87" fillId="26" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="88" fillId="27" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="89" fillId="33" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="90" fillId="27" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="83" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="86" fillId="34" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="84" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -29313,8 +29430,8 @@
           <t>CAB</t>
         </is>
       </c>
-      <c r="C35" s="38">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"CAB")</f>
+      <c r="C35" s="126">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"-")</f>
         <v/>
       </c>
       <c r="E35" s="46" t="inlineStr">
@@ -29322,8 +29439,8 @@
           <t>SEAT</t>
         </is>
       </c>
-      <c r="F35" s="47">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"SEAT")</f>
+      <c r="F35" s="127">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"-")</f>
         <v/>
       </c>
       <c r="H35" s="30" t="inlineStr">
@@ -29331,36 +29448,27 @@
           <t>AV</t>
         </is>
       </c>
-      <c r="I35" s="52">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AV")</f>
+      <c r="I35" s="128">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"-")</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="14.4" customHeight="1" s="104">
-      <c r="B36" s="126">
+      <c r="B36" s="129">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C36" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"-")</f>
-        <v/>
-      </c>
-      <c r="E36" s="126">
+      <c r="C36" s="125" t="n"/>
+      <c r="E36" s="130">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F36" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"-")</f>
-        <v/>
-      </c>
-      <c r="H36" s="126">
+      <c r="F36" s="125" t="n"/>
+      <c r="H36" s="131">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I36" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"-")</f>
-        <v/>
-      </c>
+      <c r="I36" s="125" t="n"/>
     </row>
     <row r="37" ht="32.1" customHeight="1" s="104">
       <c r="B37" s="43" t="inlineStr">
@@ -29368,8 +29476,8 @@
           <t>S/W</t>
         </is>
       </c>
-      <c r="C37" s="44">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/W")</f>
+      <c r="C37" s="132">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"-")</f>
         <v/>
       </c>
       <c r="E37" s="53" t="inlineStr">
@@ -29377,8 +29485,8 @@
           <t>S/M</t>
         </is>
       </c>
-      <c r="F37" s="54">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"S/M")</f>
+      <c r="F37" s="133">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"-")</f>
         <v/>
       </c>
       <c r="H37" s="61" t="inlineStr">
@@ -29386,36 +29494,27 @@
           <t>PAINT</t>
         </is>
       </c>
-      <c r="I37" s="62">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"PAINT")</f>
+      <c r="I37" s="134">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"-")</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="14.4" customHeight="1" s="104">
-      <c r="B38" s="126">
+      <c r="B38" s="135">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C38" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"-")</f>
-        <v/>
-      </c>
-      <c r="E38" s="126">
+      <c r="C38" s="125" t="n"/>
+      <c r="E38" s="136">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F38" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"-")</f>
-        <v/>
-      </c>
-      <c r="H38" s="126">
+      <c r="F38" s="125" t="n"/>
+      <c r="H38" s="137">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I38" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"-")</f>
-        <v/>
-      </c>
+      <c r="I38" s="125" t="n"/>
     </row>
     <row r="39" ht="32.1" customHeight="1" s="104">
       <c r="B39" s="55" t="inlineStr">
@@ -29423,8 +29522,8 @@
           <t>JOINT</t>
         </is>
       </c>
-      <c r="C39" s="56">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"JOINT")</f>
+      <c r="C39" s="138">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"-")</f>
         <v/>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -29432,8 +29531,8 @@
           <t>INSP</t>
         </is>
       </c>
-      <c r="F39" s="3">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"INSP")</f>
+      <c r="F39" s="139">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"-")</f>
         <v/>
       </c>
       <c r="H39" s="63" t="inlineStr">
@@ -29441,36 +29540,27 @@
           <t>AP</t>
         </is>
       </c>
-      <c r="I39" s="64">
-        <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!G4:G1002,"AP")</f>
+      <c r="I39" s="140">
+        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"-")</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="14.4" customHeight="1" s="104">
-      <c r="B40" s="126">
+      <c r="B40" s="141">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C40" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"-")</f>
-        <v/>
-      </c>
-      <c r="E40" s="126">
+      <c r="C40" s="125" t="n"/>
+      <c r="E40" s="129">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F40" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"-")</f>
-        <v/>
-      </c>
-      <c r="H40" s="126">
+      <c r="F40" s="125" t="n"/>
+      <c r="H40" s="131">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I40" s="127">
-        <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"-")</f>
-        <v/>
-      </c>
+      <c r="I40" s="125" t="n"/>
     </row>
     <row r="41" ht="32.1" customHeight="1" s="104"/>
   </sheetData>

</xml_diff>

<commit_message>
Add C-Check alert banner to DASHBOARD
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="84">
+  <fonts count="85">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -578,8 +578,14 @@
       <color rgb="FFE65100"/>
       <sz val="16"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill/>
     </fill>
@@ -796,6 +802,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B5E20"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -954,7 +965,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="71" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="54" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1338,12 +1349,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="84" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
     <cellStyle name="ارتباط تشعبي" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="101">
+  <dxfs count="104">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -2667,6 +2681,39 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFB71C1C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE65100"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF1B5E20"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -29074,7 +29121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="129" min="1" max="1"/>
@@ -29089,7 +29136,7 @@
     <col width="3" customWidth="1" style="129" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" s="129">
+    <row r="1" ht="28" customHeight="1" s="129">
       <c r="A1" s="121" t="inlineStr">
         <is>
           <t>📊  ASF C3-CHECK — WORK PACKAGE DASHBOARD</t>
@@ -29097,6 +29144,10 @@
       </c>
       <c r="I1" s="116">
         <f>"Day "&amp;TEXT(MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)),"0")&amp;"/36"</f>
+        <v/>
+      </c>
+      <c r="K1" s="133">
+        <f>LET(days_left, MAX(0, 36 - MAX(1, MIN(TODAY()-DATE(2026,6,8)+1,36))),open_count, COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open"),IF(TODAY()&gt;DATE(2026,7,14),"❌  C-CHECK ENDED — "&amp;open_count&amp;" Open remaining",IF(days_left&lt;5,"🔴  CRITICAL — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open",IF(days_left&lt;10,"⚠️  WARNING — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open","✅  ON TRACK — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open"))))</f>
         <v/>
       </c>
     </row>
@@ -29618,7 +29669,7 @@
     </row>
     <row r="43" ht="32.1" customHeight="1" s="129"/>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="28">
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="B22:C22"/>
@@ -29630,6 +29681,7 @@
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="H39:I39"/>
     <mergeCell ref="H25:I25"/>
+    <mergeCell ref="K1:O1"/>
     <mergeCell ref="A9:J9"/>
     <mergeCell ref="B42:C42"/>
     <mergeCell ref="E28:F28"/>
@@ -29647,6 +29699,17 @@
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="A33:J33"/>
   </mergeCells>
+  <conditionalFormatting sqref="K1:O1">
+    <cfRule type="expression" priority="1" dxfId="101">
+      <formula>OR(ISNUMBER(SEARCH("CRITICAL",K1)),ISNUMBER(SEARCH("ENDED",K1)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="102">
+      <formula>ISNUMBER(SEARCH("WARNING",K1))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="103">
+      <formula>ISNUMBER(SEARCH("ON TRACK",K1))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Add C-Check alert to row 2 in DASHBOARD
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="85">
+  <fonts count="86">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -584,6 +584,12 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="43">
     <fill>
@@ -965,7 +971,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="71" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="54" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1352,12 +1358,15 @@
     <xf numFmtId="0" fontId="84" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="85" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
     <cellStyle name="ارتباط تشعبي" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="104">
+  <dxfs count="108">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -2714,6 +2723,58 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="12"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFB71C1C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="12"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF880000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="12"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE65100"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="FFFFFFFF"/>
+        <sz val="12"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF1B5E20"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -29121,7 +29182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="129" min="1" max="1"/>
@@ -29146,528 +29207,530 @@
         <f>"Day "&amp;TEXT(MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)),"0")&amp;"/36"</f>
         <v/>
       </c>
-      <c r="K1" s="133">
-        <f>LET(days_left, MAX(0, 36 - MAX(1, MIN(TODAY()-DATE(2026,6,8)+1,36))),open_count, COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open"),IF(TODAY()&gt;DATE(2026,7,14),"❌  C-CHECK ENDED — "&amp;open_count&amp;" Open remaining",IF(days_left&lt;5,"🔴  CRITICAL — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open",IF(days_left&lt;10,"⚠️  WARNING — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open","✅  ON TRACK — "&amp;days_left&amp;" days left, "&amp;open_count&amp;" Open"))))</f>
+      <c r="K1" s="133" t="n"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" s="129">
+      <c r="A2" s="134">
+        <f>IF(TODAY()&gt;DATE(2026,7,14),"❌  C-CHECK ENDED  —  "&amp;COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open")&amp;" Open remaining",IF(MAX(0,36-MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)))&lt;5,"🔴  CRITICAL  —  "&amp;MAX(0,36-MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)))&amp;" days left  |  "&amp;COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open")&amp;" Open",IF(MAX(0,36-MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)))&lt;10,"⚠️  WARNING  —  "&amp;MAX(0,36-MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)))&amp;" days left  |  "&amp;COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open")&amp;" Open","✅  ON TRACK  —  "&amp;MAX(0,36-MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)))&amp;" days left  |  "&amp;COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open")&amp;" Open")))</f>
         <v/>
       </c>
     </row>
-    <row r="2" ht="13.9" customHeight="1" s="129">
-      <c r="A2" s="111" t="inlineStr">
+    <row r="3" ht="18" customHeight="1" s="129">
+      <c r="A3" s="111" t="inlineStr">
         <is>
           <t>All figures update automatically from ASF Tracker</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="129">
-      <c r="A3" s="109" t="inlineStr">
+    <row r="4" ht="4.15" customHeight="1" s="129">
+      <c r="A4" s="109" t="inlineStr">
         <is>
           <t xml:space="preserve">  STATUS OVERVIEW</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="4.15" customHeight="1" s="129"/>
-    <row r="5" ht="31.9" customHeight="1" s="129">
-      <c r="B5" s="64" t="inlineStr">
+    <row r="5" ht="31.9" customHeight="1" s="129"/>
+    <row r="6" ht="4.15" customHeight="1" s="129">
+      <c r="B6" s="64" t="inlineStr">
         <is>
           <t>Total Items/WOs</t>
         </is>
       </c>
-      <c r="C5" s="12">
+      <c r="C6" s="12">
         <f>COUNTIF('ASF Tracker'!B4:B1002,"&lt;&gt;")</f>
         <v/>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="F5" s="14">
+      <c r="F6" s="14">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Closed")</f>
         <v/>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>Completion</t>
         </is>
       </c>
-      <c r="I5" s="16">
+      <c r="I6" s="16">
         <f>TEXT(IFERROR(COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Closed")/COUNTIF('ASF Tracker'!B4:B1002,"&lt;&gt;"),0),"0%")</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="4.15" customHeight="1" s="129"/>
-    <row r="7" ht="31.9" customHeight="1" s="129">
-      <c r="B7" s="65" t="inlineStr">
+    <row r="7" ht="31.9" customHeight="1" s="129"/>
+    <row r="8" ht="4.15" customHeight="1" s="129">
+      <c r="B8" s="65" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="C7" s="17">
+      <c r="C8" s="17">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Open")</f>
         <v/>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="F7" s="19">
+      <c r="F8" s="19">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"In Progress")</f>
         <v/>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>Deferred / Hold</t>
         </is>
       </c>
-      <c r="I7" s="21">
+      <c r="I8" s="21">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"Deferred")+COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!E4:E1002,"On Hold")</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="4.15" customHeight="1" s="129"/>
-    <row r="9" ht="18" customHeight="1" s="129">
-      <c r="A9" s="124" t="inlineStr">
+    <row r="9" ht="18" customHeight="1" s="129"/>
+    <row r="10" ht="4.15" customHeight="1" s="129">
+      <c r="A10" s="124" t="inlineStr">
         <is>
           <t xml:space="preserve">  PRIORITY ALERTS</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="4.15" customHeight="1" s="129"/>
-    <row r="11" ht="31.9" customHeight="1" s="129">
-      <c r="B11" s="66" t="inlineStr">
+    <row r="11" ht="31.9" customHeight="1" s="129"/>
+    <row r="12" ht="4.15" customHeight="1" s="129">
+      <c r="B12" s="66" t="inlineStr">
         <is>
           <t>AOG</t>
         </is>
       </c>
-      <c r="C11" s="22">
+      <c r="C12" s="22">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!F4:F1002,"AOG")</f>
         <v/>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F11" s="19">
+      <c r="F12" s="19">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!F4:F1002,"Critical")</f>
         <v/>
       </c>
-      <c r="H11" s="23" t="inlineStr">
+      <c r="H12" s="23" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I11" s="24">
+      <c r="I12" s="24">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!F4:F1002,"High")</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="4.15" customHeight="1" s="129"/>
-    <row r="13" ht="18" customHeight="1" s="129">
-      <c r="A13" s="109" t="inlineStr">
+    <row r="13" ht="18" customHeight="1" s="129"/>
+    <row r="14" ht="4.15" customHeight="1" s="129">
+      <c r="A14" s="109" t="inlineStr">
         <is>
           <t xml:space="preserve">  PARTS REQUIREMENTS  (count of WOs with each status)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="4.15" customHeight="1" s="129"/>
-    <row r="15" ht="31.9" customHeight="1" s="129">
-      <c r="B15" s="25" t="inlineStr">
+    <row r="15" ht="31.9" customHeight="1" s="129"/>
+    <row r="16" ht="4.15" customHeight="1" s="129">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Requested</t>
         </is>
       </c>
-      <c r="C15" s="26">
+      <c r="C16" s="26">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"Requested")</f>
         <v/>
       </c>
-      <c r="E15" s="27" t="inlineStr">
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>Requested – CR</t>
         </is>
       </c>
-      <c r="F15" s="28">
+      <c r="F16" s="28">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"Requested - CR")</f>
         <v/>
       </c>
-      <c r="H15" s="29" t="inlineStr">
+      <c r="H16" s="29" t="inlineStr">
         <is>
           <t>Requested – R</t>
         </is>
       </c>
-      <c r="I15" s="30">
+      <c r="I16" s="30">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"Requested - R")</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="4.15" customHeight="1" s="129"/>
-    <row r="17" ht="31.9" customHeight="1" s="129">
-      <c r="B17" s="69" t="inlineStr">
+    <row r="17" ht="31.9" customHeight="1" s="129"/>
+    <row r="18" ht="4.15" customHeight="1" s="129">
+      <c r="B18" s="69" t="inlineStr">
         <is>
           <t>Pending - Require Evaluation</t>
         </is>
       </c>
-      <c r="C17" s="31">
+      <c r="C18" s="31">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"Pending EVAL")</f>
         <v/>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>N/R  (not required)</t>
         </is>
       </c>
-      <c r="F17" s="14">
+      <c r="F18" s="14">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"N/R")</f>
         <v/>
       </c>
-      <c r="H17" s="32" t="inlineStr">
+      <c r="H18" s="32" t="inlineStr">
         <is>
           <t>N/A (Not available)</t>
         </is>
       </c>
-      <c r="I17" s="33">
+      <c r="I18" s="33">
         <f>COUNTIFS('ASF Tracker'!B4:B1002,"&lt;&gt;",'ASF Tracker'!H4:H1002,"N/A")</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="4.15" customHeight="1" s="129"/>
-    <row r="19" ht="18" customHeight="1" s="129">
-      <c r="A19" s="109" t="inlineStr">
+    <row r="19" ht="18" customHeight="1" s="129"/>
+    <row r="20" ht="4.15" customHeight="1" s="129">
+      <c r="A20" s="109" t="inlineStr">
         <is>
           <t xml:space="preserve">  BY CATEGORY</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="4.15" customHeight="1" s="129"/>
-    <row r="21" ht="31.9" customHeight="1" s="129">
-      <c r="B21" s="34" t="inlineStr">
+    <row r="21" ht="31.9" customHeight="1" s="129"/>
+    <row r="22" ht="14.45" customHeight="1" s="129">
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>TASK CARD</t>
         </is>
       </c>
-      <c r="C21" s="35">
+      <c r="C22" s="35">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD"),"-")</f>
         <v/>
       </c>
-      <c r="E21" s="36" t="inlineStr">
+      <c r="E22" s="36" t="inlineStr">
         <is>
           <t>LAVATORY</t>
         </is>
       </c>
-      <c r="F21" s="37">
+      <c r="F22" s="37">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY"),"-")</f>
         <v/>
       </c>
-      <c r="H21" s="38" t="inlineStr">
+      <c r="H22" s="38" t="inlineStr">
         <is>
           <t>GALLEY</t>
         </is>
       </c>
-      <c r="I21" s="39">
+      <c r="I22" s="39">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="14.45" customHeight="1" s="129">
-      <c r="B22" s="119">
+    <row r="23" ht="4.15" customHeight="1" s="129">
+      <c r="B23" s="119">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C22" s="132" t="n"/>
-      <c r="E22" s="110">
+      <c r="C23" s="132" t="n"/>
+      <c r="E23" s="110">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F22" s="132" t="n"/>
-      <c r="H22" s="113">
+      <c r="F23" s="132" t="n"/>
+      <c r="H23" s="113">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I22" s="132" t="n"/>
-    </row>
-    <row r="23" ht="4.15" customHeight="1" s="129">
-      <c r="B23" s="54" t="n"/>
-      <c r="E23" s="54" t="n"/>
-      <c r="H23" s="54" t="n"/>
+      <c r="I23" s="132" t="n"/>
     </row>
     <row r="24" ht="31.9" customHeight="1" s="129">
-      <c r="B24" s="40" t="inlineStr">
+      <c r="B24" s="54" t="n"/>
+      <c r="E24" s="54" t="n"/>
+      <c r="H24" s="54" t="n"/>
+    </row>
+    <row r="25" ht="14.45" customHeight="1" s="129">
+      <c r="B25" s="40" t="inlineStr">
         <is>
           <t>GENERAL CABIN</t>
         </is>
       </c>
-      <c r="C24" s="41">
+      <c r="C25" s="41">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1002,"Closed",'ASF Tracker'!$B$4:$B$1002,"&lt;&gt;")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$B$4:$B$1002,"&lt;&gt;"),"-")</f>
         <v/>
       </c>
-      <c r="E24" s="42" t="inlineStr">
+      <c r="E25" s="42" t="inlineStr">
         <is>
           <t>TEDLAR/SIDEWALL</t>
         </is>
       </c>
-      <c r="F24" s="43">
+      <c r="F25" s="43">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL"),"-")</f>
         <v/>
       </c>
-      <c r="H24" s="67" t="inlineStr">
+      <c r="H25" s="67" t="inlineStr">
         <is>
           <t>PAX SEAT</t>
         </is>
       </c>
-      <c r="I24" s="44">
+      <c r="I25" s="44">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="25" ht="14.45" customHeight="1" s="129">
-      <c r="B25" s="115">
+    <row r="26" ht="4.15" customHeight="1" s="129">
+      <c r="B26" s="115">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1002,"Closed",'ASF Tracker'!$B$4:$B$1002,"&lt;&gt;")/COUNTIFS('ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$B$4:$B$1002,"&lt;&gt;"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C25" s="132" t="n"/>
-      <c r="E25" s="117">
+      <c r="C26" s="132" t="n"/>
+      <c r="E26" s="117">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F25" s="132" t="n"/>
-      <c r="H25" s="120">
+      <c r="F26" s="132" t="n"/>
+      <c r="H26" s="120">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I25" s="132" t="n"/>
-    </row>
-    <row r="26" ht="4.15" customHeight="1" s="129">
-      <c r="B26" s="54" t="n"/>
-      <c r="E26" s="54" t="n"/>
-      <c r="H26" s="54" t="n"/>
+      <c r="I26" s="132" t="n"/>
     </row>
     <row r="27" ht="31.9" customHeight="1" s="129">
-      <c r="B27" s="45" t="inlineStr">
+      <c r="B27" s="54" t="n"/>
+      <c r="E27" s="54" t="n"/>
+      <c r="H27" s="54" t="n"/>
+    </row>
+    <row r="28" ht="14.45" customHeight="1" s="129">
+      <c r="B28" s="45" t="inlineStr">
         <is>
           <t>PAX DOORS</t>
         </is>
       </c>
-      <c r="C27" s="46">
+      <c r="C28" s="46">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS"),"-")</f>
         <v/>
       </c>
-      <c r="E27" s="47" t="inlineStr">
+      <c r="E28" s="47" t="inlineStr">
         <is>
           <t>F/A SEAT</t>
         </is>
       </c>
-      <c r="F27" s="48">
+      <c r="F28" s="48">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT"),"-")</f>
         <v/>
       </c>
-      <c r="H27" s="55" t="inlineStr">
+      <c r="H28" s="55" t="inlineStr">
         <is>
           <t>OTHERS</t>
         </is>
       </c>
-      <c r="I27" s="56">
+      <c r="I28" s="56">
         <f>IFERROR((COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$E$4:$E$1002,"Closed")-(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"OFAR/OFCR",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1002,"Closed")))&amp;" / "&amp;(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;")-(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"OFAR/OFCR")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK"))),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="28" ht="14.45" customHeight="1" s="129">
-      <c r="B28" s="112">
+    <row r="29" ht="4.15" customHeight="1" s="129">
+      <c r="B29" s="112">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C28" s="132" t="n"/>
-      <c r="E28" s="125">
+      <c r="C29" s="132" t="n"/>
+      <c r="E29" s="125">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F28" s="132" t="n"/>
-      <c r="H28" s="114">
+      <c r="F29" s="132" t="n"/>
+      <c r="H29" s="114">
         <f>IFERROR("Completion: "&amp;TEXT(((COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$E$4:$E$1002,"Closed")-(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"OFAR/OFCR",'ASF Tracker'!$E$4:$E$1002,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1002,"Closed"))))/((COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;")-(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TASK CARD")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"LAVATORY")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GALLEY")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"GENERAL CABIN")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"TEDLAR/SIDEWALL")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"PAX DOORS")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"F/A SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"OFAR/OFCR")+COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK")))),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I28" s="132" t="n"/>
-    </row>
-    <row r="29" ht="4.15" customHeight="1" s="129">
-      <c r="B29" s="54" t="n"/>
-      <c r="E29" s="54" t="n"/>
+      <c r="I29" s="132" t="n"/>
     </row>
     <row r="30" ht="31.9" customHeight="1" s="129">
-      <c r="B30" s="49" t="inlineStr">
+      <c r="B30" s="54" t="n"/>
+      <c r="E30" s="54" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="49" t="inlineStr">
         <is>
           <t>FLIGHT DECK</t>
         </is>
       </c>
-      <c r="C30" s="50">
+      <c r="C31" s="50">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="120">
+    <row r="32" ht="4.15" customHeight="1" s="129">
+      <c r="B32" s="120">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1002,"FLIGHT DECK"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C31" s="132" t="n"/>
-    </row>
-    <row r="32" ht="4.15" customHeight="1" s="129"/>
-    <row r="33" ht="18" customHeight="1" s="129">
-      <c r="A33" s="109" t="inlineStr">
+      <c r="C32" s="132" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="129"/>
+    <row r="34" ht="4.15" customHeight="1" s="129">
+      <c r="A34" s="109" t="inlineStr">
         <is>
           <t xml:space="preserve">  SPECIALTY</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="4.15" customHeight="1" s="129"/>
-    <row r="35" ht="32.1" customHeight="1" s="129">
-      <c r="B35" s="36" t="inlineStr">
+    <row r="35" ht="32.1" customHeight="1" s="129"/>
+    <row r="36" ht="14.45" customHeight="1" s="129">
+      <c r="B36" s="36" t="inlineStr">
         <is>
           <t>CABIN</t>
         </is>
       </c>
-      <c r="C35" s="92">
+      <c r="C36" s="92">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"-")</f>
         <v/>
       </c>
-      <c r="E35" s="45" t="inlineStr">
+      <c r="E36" s="45" t="inlineStr">
         <is>
           <t>SEAT SHOP</t>
         </is>
       </c>
-      <c r="F35" s="93">
+      <c r="F36" s="93">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"-")</f>
         <v/>
       </c>
-      <c r="H35" s="29" t="inlineStr">
+      <c r="H36" s="29" t="inlineStr">
         <is>
           <t>AV/FOMAX</t>
         </is>
       </c>
-      <c r="I35" s="94">
+      <c r="I36" s="94">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="14.45" customHeight="1" s="129">
-      <c r="B36" s="110">
+    <row r="37" ht="3.75" customHeight="1" s="129">
+      <c r="B37" s="110">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"CAB"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C36" s="132" t="n"/>
-      <c r="E36" s="112">
+      <c r="C37" s="132" t="n"/>
+      <c r="E37" s="112">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"SEAT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F36" s="132" t="n"/>
-      <c r="H36" s="115">
+      <c r="F37" s="132" t="n"/>
+      <c r="H37" s="115">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AV"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I36" s="132" t="n"/>
-    </row>
-    <row r="37" ht="3.75" customHeight="1" s="129">
-      <c r="B37" s="54" t="n"/>
-      <c r="E37" s="54" t="n"/>
-      <c r="H37" s="54" t="n"/>
+      <c r="I37" s="132" t="n"/>
     </row>
     <row r="38" ht="32.1" customHeight="1" s="129">
-      <c r="B38" s="42" t="inlineStr">
+      <c r="B38" s="54" t="n"/>
+      <c r="E38" s="54" t="n"/>
+      <c r="H38" s="54" t="n"/>
+    </row>
+    <row r="39" ht="14.45" customHeight="1" s="129">
+      <c r="B39" s="42" t="inlineStr">
         <is>
           <t>SIDEWALL</t>
         </is>
       </c>
-      <c r="C38" s="95">
+      <c r="C39" s="95">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"-")</f>
         <v/>
       </c>
-      <c r="E38" s="51" t="inlineStr">
+      <c r="E39" s="51" t="inlineStr">
         <is>
           <t>S/M</t>
         </is>
       </c>
-      <c r="F38" s="96">
+      <c r="F39" s="96">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"-")</f>
         <v/>
       </c>
-      <c r="H38" s="57" t="inlineStr">
+      <c r="H39" s="57" t="inlineStr">
         <is>
           <t>PAINT</t>
         </is>
       </c>
-      <c r="I38" s="97">
+      <c r="I39" s="97">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="14.45" customHeight="1" s="129">
-      <c r="B39" s="117">
+    <row r="40" ht="3.75" customHeight="1" s="129">
+      <c r="B40" s="117">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/W"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C39" s="132" t="n"/>
-      <c r="E39" s="122">
+      <c r="C40" s="132" t="n"/>
+      <c r="E40" s="122">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"S/M"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F39" s="132" t="n"/>
-      <c r="H39" s="123">
+      <c r="F40" s="132" t="n"/>
+      <c r="H40" s="123">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"PAINT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I39" s="132" t="n"/>
-    </row>
-    <row r="40" ht="3.75" customHeight="1" s="129">
-      <c r="B40" s="54" t="n"/>
-      <c r="E40" s="54" t="n"/>
-      <c r="H40" s="54" t="n"/>
+      <c r="I40" s="132" t="n"/>
     </row>
     <row r="41" ht="32.1" customHeight="1" s="129">
-      <c r="B41" s="52" t="inlineStr">
+      <c r="B41" s="54" t="n"/>
+      <c r="E41" s="54" t="n"/>
+      <c r="H41" s="54" t="n"/>
+    </row>
+    <row r="42" ht="14.45" customHeight="1" s="129">
+      <c r="B42" s="52" t="inlineStr">
         <is>
           <t>JOINT</t>
         </is>
       </c>
-      <c r="C41" s="98">
+      <c r="C42" s="98">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"-")</f>
         <v/>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>INSP</t>
         </is>
       </c>
-      <c r="F41" s="99">
+      <c r="F42" s="99">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"-")</f>
         <v/>
       </c>
-      <c r="H41" s="58" t="inlineStr">
+      <c r="H42" s="58" t="inlineStr">
         <is>
           <t>A/P</t>
         </is>
       </c>
-      <c r="I41" s="100">
+      <c r="I42" s="100">
         <f>IFERROR(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")&amp;" / "&amp;COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"-")</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="14.45" customHeight="1" s="129">
-      <c r="B42" s="122">
+    <row r="43" ht="32.1" customHeight="1" s="129">
+      <c r="B43" s="122">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"JOINT"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="C42" s="132" t="n"/>
-      <c r="E42" s="118">
+      <c r="C43" s="132" t="n"/>
+      <c r="E43" s="118">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"INSP"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="F42" s="132" t="n"/>
-      <c r="H42" s="108">
+      <c r="F43" s="132" t="n"/>
+      <c r="H43" s="108">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP",'ASF Tracker'!$E$4:$E$1002,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1002,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1002,"AP"),"0%"),"-")</f>
         <v/>
       </c>
-      <c r="I42" s="132" t="n"/>
-    </row>
-    <row r="43" ht="32.1" customHeight="1" s="129"/>
+      <c r="I43" s="132" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="28">
     <mergeCell ref="B25:C25"/>
@@ -29708,6 +29771,20 @@
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="103">
       <formula>ISNUMBER(SEARCH("ON TRACK",K1))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:J2">
+    <cfRule type="expression" priority="4" dxfId="104">
+      <formula>ISNUMBER(SEARCH("CRITICAL",A2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="105">
+      <formula>ISNUMBER(SEARCH("ENDED",A2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="106">
+      <formula>ISNUMBER(SEARCH("WARNING",A2))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="107">
+      <formula>ISNUMBER(SEARCH("ON TRACK",A2))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ASF Tracker: close new + reopen missing from file
</commit_message>
<xml_diff>
--- a/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
+++ b/uploads/ASF_CABIN_WP_TRACKER_updated.xlsx
@@ -1246,34 +1246,13 @@
     <xf numFmtId="0" fontId="71" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="34" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="23" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="24" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="22" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="59" fillId="32" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="25" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="64" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="56" fillId="26" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="25" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="56" fillId="28" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1291,6 +1270,9 @@
     <xf numFmtId="0" fontId="56" fillId="27" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="56" fillId="33" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1298,6 +1280,24 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="56" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="34" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="23" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="24" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="22" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="32" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="62" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2770,6 +2770,7 @@
       <filters>
         <filter val="CAB"/>
         <filter val="JOINT"/>
+        <filter val="S/M"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -3033,7 +3034,7 @@
     <row r="2" ht="19.9" customHeight="1" s="125">
       <c r="A2" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">UPDATED: 07 JULY -- DAY SHIFT </t>
+          <t xml:space="preserve">UPDATED: 08 JULY -- DAY SHIFT </t>
         </is>
       </c>
       <c r="B2" s="126" t="n"/>
@@ -3223,7 +3224,7 @@
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -3249,7 +3250,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" s="125">
+    <row r="7" hidden="1" ht="18" customHeight="1" s="125">
       <c r="A7" s="68" t="n">
         <v>24</v>
       </c>
@@ -3406,7 +3407,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="125">
+    <row r="10" hidden="1" ht="18" customHeight="1" s="125">
       <c r="A10" s="68" t="n">
         <v>27</v>
       </c>
@@ -3482,7 +3483,7 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
@@ -3502,7 +3503,7 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>I/W</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
@@ -3866,7 +3867,7 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -3880,7 +3881,11 @@
         </is>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="9" t="n"/>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>TO BE CLOSED</t>
+        </is>
+      </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -4038,7 +4043,7 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -4052,7 +4057,11 @@
         </is>
       </c>
       <c r="H23" s="10" t="n"/>
-      <c r="I23" s="9" t="n"/>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>TO BE CLOSED</t>
+        </is>
+      </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -5268,7 +5277,7 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr">
@@ -6157,7 +6166,7 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr">
@@ -6173,7 +6182,7 @@
       <c r="H72" s="10" t="n"/>
       <c r="I72" s="9" t="inlineStr">
         <is>
-          <t>R/R FROM CATRION</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr">
@@ -6715,7 +6724,7 @@
       </c>
       <c r="K84" s="9" t="n"/>
     </row>
-    <row r="85" hidden="1" ht="18" customHeight="1" s="125">
+    <row r="85" ht="18" customHeight="1" s="125">
       <c r="A85" s="68" t="n">
         <v>341</v>
       </c>
@@ -6734,7 +6743,7 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr">
@@ -6820,7 +6829,7 @@
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F87" s="9" t="inlineStr">
@@ -6918,7 +6927,11 @@
         </is>
       </c>
       <c r="H89" s="10" t="n"/>
-      <c r="I89" s="9" t="n"/>
+      <c r="I89" s="9" t="inlineStr">
+        <is>
+          <t>TO BE CLOSED</t>
+        </is>
+      </c>
       <c r="J89" s="9" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -7039,7 +7052,7 @@
       </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F92" s="9" t="inlineStr">
@@ -7700,7 +7713,7 @@
       </c>
       <c r="E107" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F107" s="9" t="inlineStr">
@@ -7720,7 +7733,7 @@
       </c>
       <c r="I107" s="9" t="inlineStr">
         <is>
-          <t>P/S 4467481</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J107" s="9" t="inlineStr">
@@ -7755,7 +7768,7 @@
       </c>
       <c r="E108" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F108" s="9" t="inlineStr">
@@ -7771,7 +7784,7 @@
       <c r="H108" s="10" t="n"/>
       <c r="I108" s="9" t="inlineStr">
         <is>
-          <t>I/W</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J108" s="9" t="inlineStr">
@@ -9055,7 +9068,7 @@
         </is>
       </c>
     </row>
-    <row r="137" hidden="1" ht="15.6" customHeight="1" s="125">
+    <row r="137" ht="15.6" customHeight="1" s="125">
       <c r="A137" s="68" t="inlineStr">
         <is>
           <t>506</t>
@@ -9127,7 +9140,7 @@
       </c>
       <c r="E138" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F138" s="9" t="inlineStr">
@@ -9143,7 +9156,7 @@
       <c r="H138" s="10" t="n"/>
       <c r="I138" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">S/M REPAIR C/W </t>
+          <t>TO DO</t>
         </is>
       </c>
       <c r="J138" s="9" t="inlineStr">
@@ -9315,7 +9328,7 @@
       </c>
       <c r="E142" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
@@ -9344,7 +9357,7 @@
       <c r="B143" s="63" t="n">
         <v>32395971</v>
       </c>
-      <c r="C143" s="7" t="inlineStr">
+      <c r="C143" s="81" t="inlineStr">
         <is>
           <t>CCC-32S (03) / A32S CABIN CRITICAL CHECK</t>
         </is>
@@ -9385,7 +9398,7 @@
       <c r="B144" s="63" t="n">
         <v>32349954</v>
       </c>
-      <c r="C144" s="7" t="inlineStr">
+      <c r="C144" s="81" t="inlineStr">
         <is>
           <t>DCC-32S (11) / DCC A32S DAILY CABIN CHECK</t>
         </is>
@@ -9508,7 +9521,7 @@
       <c r="B147" s="63" t="n">
         <v>32258914</v>
       </c>
-      <c r="C147" s="7" t="inlineStr">
+      <c r="C147" s="81" t="inlineStr">
         <is>
           <t>W_N/WEEKLY CHECK</t>
         </is>
@@ -9551,7 +9564,7 @@
           <t>ISC-32S</t>
         </is>
       </c>
-      <c r="C148" s="7" t="inlineStr">
+      <c r="C148" s="81" t="inlineStr">
         <is>
           <t>ISC-32S (13) / 32S IN-SERVEICE-CHECK (ISC)</t>
         </is>
@@ -9653,7 +9666,7 @@
       </c>
       <c r="E150" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
@@ -9827,7 +9840,7 @@
           <t>WEEKLY-32S</t>
         </is>
       </c>
-      <c r="C154" s="7" t="inlineStr">
+      <c r="C154" s="81" t="inlineStr">
         <is>
           <t>WEEKLY-32S (04) / WEEKLY 32S CHECK</t>
         </is>
@@ -10170,7 +10183,7 @@
       </c>
       <c r="E161" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F161" s="9" t="inlineStr">
@@ -12878,7 +12891,7 @@
       </c>
       <c r="E217" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F217" s="9" t="inlineStr">
@@ -12919,7 +12932,7 @@
       </c>
       <c r="E218" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F218" s="9" t="inlineStr">
@@ -12968,7 +12981,7 @@
       </c>
       <c r="E219" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F219" s="9" t="inlineStr">
@@ -13017,7 +13030,7 @@
       </c>
       <c r="E220" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F220" s="9" t="inlineStr">
@@ -13066,7 +13079,7 @@
       </c>
       <c r="E221" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F221" s="9" t="inlineStr">
@@ -13409,7 +13422,7 @@
       </c>
       <c r="E228" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F228" s="9" t="inlineStr">
@@ -13458,7 +13471,7 @@
       </c>
       <c r="E229" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F229" s="9" t="inlineStr">
@@ -13507,7 +13520,7 @@
       </c>
       <c r="E230" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F230" s="9" t="inlineStr">
@@ -13556,7 +13569,7 @@
       </c>
       <c r="E231" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F231" s="9" t="inlineStr">
@@ -13605,7 +13618,7 @@
       </c>
       <c r="E232" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F232" s="9" t="inlineStr">
@@ -13654,7 +13667,7 @@
       </c>
       <c r="E233" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F233" s="9" t="inlineStr">
@@ -13703,7 +13716,7 @@
       </c>
       <c r="E234" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F234" s="9" t="inlineStr">
@@ -13752,7 +13765,7 @@
       </c>
       <c r="E235" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F235" s="9" t="inlineStr">
@@ -13801,7 +13814,7 @@
       </c>
       <c r="E236" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F236" s="9" t="inlineStr">
@@ -13850,7 +13863,7 @@
       </c>
       <c r="E237" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F237" s="9" t="inlineStr">
@@ -13948,7 +13961,7 @@
       </c>
       <c r="E239" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F239" s="9" t="inlineStr">
@@ -14552,7 +14565,7 @@
       </c>
       <c r="E251" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F251" s="9" t="inlineStr">
@@ -14736,7 +14749,7 @@
       </c>
       <c r="E255" s="9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F255" s="9" t="inlineStr">
@@ -15422,7 +15435,7 @@
       </c>
       <c r="E269" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F269" s="9" t="inlineStr">
@@ -15475,7 +15488,7 @@
       </c>
       <c r="E270" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F270" s="9" t="inlineStr">
@@ -15581,7 +15594,7 @@
       </c>
       <c r="E272" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F272" s="9" t="inlineStr">
@@ -15634,7 +15647,7 @@
       </c>
       <c r="E273" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F273" s="9" t="inlineStr">
@@ -16527,7 +16540,7 @@
       </c>
       <c r="E290" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F290" s="9" t="inlineStr">
@@ -16947,7 +16960,7 @@
       </c>
       <c r="E298" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F298" s="9" t="inlineStr">
@@ -17388,7 +17401,7 @@
       </c>
       <c r="E307" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F307" s="9" t="inlineStr">
@@ -17433,7 +17446,7 @@
       </c>
       <c r="E308" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F308" s="9" t="inlineStr">
@@ -17562,7 +17575,7 @@
       </c>
       <c r="E311" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F311" s="9" t="inlineStr">
@@ -17906,7 +17919,7 @@
       </c>
       <c r="E319" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F319" s="9" t="inlineStr">
@@ -18193,7 +18206,7 @@
       </c>
       <c r="E326" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F326" s="9" t="inlineStr">
@@ -18234,7 +18247,7 @@
       </c>
       <c r="E327" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F327" s="9" t="inlineStr">
@@ -18275,7 +18288,7 @@
       </c>
       <c r="E328" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F328" s="9" t="inlineStr">
@@ -18648,7 +18661,7 @@
       </c>
       <c r="E337" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F337" s="9" t="inlineStr">
@@ -18959,7 +18972,7 @@
       </c>
       <c r="E344" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F344" s="9" t="inlineStr">
@@ -19086,7 +19099,7 @@
       </c>
       <c r="E347" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F347" s="9" t="inlineStr">
@@ -19102,7 +19115,7 @@
       <c r="H347" s="10" t="n"/>
       <c r="I347" s="9" t="inlineStr">
         <is>
-          <t>OPS AND CLOSE UP TO DO (AVIO)</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J347" s="9" t="inlineStr">
@@ -19937,7 +19950,7 @@
       </c>
       <c r="E366" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F366" s="9" t="inlineStr">
@@ -19994,7 +20007,11 @@
           <t>N/R</t>
         </is>
       </c>
-      <c r="I367" s="9" t="n"/>
+      <c r="I367" s="9" t="inlineStr">
+        <is>
+          <t>INSP</t>
+        </is>
+      </c>
       <c r="J367" s="9" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -20133,7 +20150,7 @@
       </c>
       <c r="I370" s="9" t="inlineStr">
         <is>
-          <t>DAY SHIFT</t>
+          <t>INSP</t>
         </is>
       </c>
       <c r="J370" s="9" t="inlineStr">
@@ -20301,7 +20318,7 @@
       </c>
       <c r="E374" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F374" s="9" t="inlineStr">
@@ -20321,7 +20338,7 @@
       </c>
       <c r="I374" s="9" t="inlineStr">
         <is>
-          <t>TORQUE AND OPS</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J374" s="9" t="inlineStr">
@@ -20657,7 +20674,7 @@
       </c>
       <c r="E382" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F382" s="9" t="inlineStr">
@@ -20673,7 +20690,7 @@
       <c r="H382" s="10" t="n"/>
       <c r="I382" s="9" t="inlineStr">
         <is>
-          <t>OPS AND CLOSE UP TO DO (AVIO)</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J382" s="9" t="inlineStr">
@@ -20702,7 +20719,7 @@
       </c>
       <c r="E383" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F383" s="9" t="inlineStr">
@@ -20718,7 +20735,7 @@
       <c r="H383" s="10" t="n"/>
       <c r="I383" s="9" t="inlineStr">
         <is>
-          <t>OPS AND CLOSE UP TO DO (AVIO)</t>
+          <t>TO BE CLOSED</t>
         </is>
       </c>
       <c r="J383" s="9" t="inlineStr">
@@ -20788,7 +20805,7 @@
       </c>
       <c r="E385" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F385" s="9" t="inlineStr">
@@ -20829,7 +20846,7 @@
       </c>
       <c r="E386" s="9" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F386" s="9" t="inlineStr">
@@ -20847,8 +20864,16 @@
           <t>Requested - CR</t>
         </is>
       </c>
-      <c r="I386" s="9" t="n"/>
-      <c r="J386" s="9" t="n"/>
+      <c r="I386" s="9" t="inlineStr">
+        <is>
+          <t>TO BE CLOSED</t>
+        </is>
+      </c>
+      <c r="J386" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K386" s="9" t="n"/>
     </row>
     <row r="387" hidden="1" ht="18" customHeight="1" s="125">
@@ -29773,25 +29798,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" s="125">
-      <c r="A1" s="117" t="inlineStr">
+      <c r="A1" s="110" t="inlineStr">
         <is>
           <t>📊  ASF C3-CHECK — WORK PACKAGE DASHBOARD</t>
         </is>
       </c>
-      <c r="I1" s="112">
+      <c r="I1" s="104">
         <f>"Day "&amp;TEXT(MAX(1,MIN(TODAY()-DATE(2026,6,8)+1,36)),"0")&amp;"/36"</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="13.9" customHeight="1" s="125">
-      <c r="A2" s="107" t="inlineStr">
+      <c r="A2" s="118" t="inlineStr">
         <is>
           <t>All figures update automatically from ASF Tracker</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1" s="125">
-      <c r="A3" s="105" t="inlineStr">
+      <c r="A3" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">  STATUS OVERVIEW</t>
         </is>
@@ -29859,7 +29884,7 @@
     </row>
     <row r="8" ht="4.15" customHeight="1" s="125"/>
     <row r="9" ht="18" customHeight="1" s="125">
-      <c r="A9" s="120" t="inlineStr">
+      <c r="A9" s="114" t="inlineStr">
         <is>
           <t xml:space="preserve">  PRIORITY ALERTS</t>
         </is>
@@ -29897,7 +29922,7 @@
     </row>
     <row r="12" ht="4.15" customHeight="1" s="125"/>
     <row r="13" ht="18" customHeight="1" s="125">
-      <c r="A13" s="105" t="inlineStr">
+      <c r="A13" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">  PARTS REQUIREMENTS  (count of WOs with each status)</t>
         </is>
@@ -29965,7 +29990,7 @@
     </row>
     <row r="18" ht="4.15" customHeight="1" s="125"/>
     <row r="19" ht="18" customHeight="1" s="125">
-      <c r="A19" s="105" t="inlineStr">
+      <c r="A19" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">  BY CATEGORY</t>
         </is>
@@ -30002,17 +30027,17 @@
       </c>
     </row>
     <row r="22" ht="14.45" customHeight="1" s="125">
-      <c r="B22" s="115">
+      <c r="B22" s="108">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TASK CARD",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TASK CARD"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C22" s="128" t="n"/>
-      <c r="E22" s="106">
+      <c r="E22" s="117">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"LAVATORY",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"LAVATORY"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F22" s="128" t="n"/>
-      <c r="H22" s="109">
+      <c r="H22" s="120">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GALLEY",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GALLEY"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30053,17 +30078,17 @@
       </c>
     </row>
     <row r="25" ht="14.45" customHeight="1" s="125">
-      <c r="B25" s="111">
+      <c r="B25" s="106">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$D$4:$D$1004,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1004,"Closed",'ASF Tracker'!$B$4:$B$1004,"&lt;&gt;")/COUNTIFS('ASF Tracker'!$D$4:$D$1004,"GENERAL CABIN",'ASF Tracker'!$B$4:$B$1004,"&lt;&gt;"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C25" s="128" t="n"/>
-      <c r="E25" s="113">
+      <c r="E25" s="105">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TEDLAR/SIDEWALL"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F25" s="128" t="n"/>
-      <c r="H25" s="116">
+      <c r="H25" s="109">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX SEAT",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX SEAT"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30104,17 +30129,17 @@
       </c>
     </row>
     <row r="28" ht="14.45" customHeight="1" s="125">
-      <c r="B28" s="108">
+      <c r="B28" s="119">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX DOORS",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX DOORS"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C28" s="128" t="n"/>
-      <c r="E28" s="121">
+      <c r="E28" s="115">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"F/A SEAT",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"F/A SEAT"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F28" s="128" t="n"/>
-      <c r="H28" s="110">
+      <c r="H28" s="121">
         <f>IFERROR("Completion: "&amp;TEXT(((COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$E$4:$E$1004,"Closed")-(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TASK CARD",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"LAVATORY",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GALLEY",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GENERAL CABIN",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TEDLAR/SIDEWALL",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX SEAT",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX DOORS",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"F/A SEAT",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"OFAR/OFCR",'ASF Tracker'!$E$4:$E$1004,"Closed")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1004,"Closed"))))/((COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;")-(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TASK CARD")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"LAVATORY")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GALLEY")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"GENERAL CABIN")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"TEDLAR/SIDEWALL")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"PAX DOORS")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"F/A SEAT")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"OFAR/OFCR")+COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"FLIGHT DECK")))),"0%"),"-")</f>
         <v/>
       </c>
@@ -30136,7 +30161,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="116">
+      <c r="B31" s="109">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"FLIGHT DECK",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$D$4:$D$1004,"FLIGHT DECK"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30144,7 +30169,7 @@
     </row>
     <row r="32" ht="4.15" customHeight="1" s="125"/>
     <row r="33" ht="18" customHeight="1" s="125">
-      <c r="A33" s="105" t="inlineStr">
+      <c r="A33" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">  SPECIALTY</t>
         </is>
@@ -30181,17 +30206,17 @@
       </c>
     </row>
     <row r="36" ht="14.45" customHeight="1" s="125">
-      <c r="B36" s="106">
+      <c r="B36" s="117">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"CAB",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"CAB"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C36" s="128" t="n"/>
-      <c r="E36" s="108">
+      <c r="E36" s="119">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"SEAT",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"SEAT"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F36" s="128" t="n"/>
-      <c r="H36" s="111">
+      <c r="H36" s="106">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"AV",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"AV"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30232,17 +30257,17 @@
       </c>
     </row>
     <row r="39" ht="14.45" customHeight="1" s="125">
-      <c r="B39" s="113">
+      <c r="B39" s="105">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"S/W",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"S/W"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C39" s="128" t="n"/>
-      <c r="E39" s="118">
+      <c r="E39" s="111">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"S/M",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"S/M"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F39" s="128" t="n"/>
-      <c r="H39" s="119">
+      <c r="H39" s="113">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"PAINT",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"PAINT"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30283,17 +30308,17 @@
       </c>
     </row>
     <row r="42" ht="14.45" customHeight="1" s="125">
-      <c r="B42" s="118">
+      <c r="B42" s="111">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"JOINT",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"JOINT"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="C42" s="128" t="n"/>
-      <c r="E42" s="114">
+      <c r="E42" s="107">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"INSP",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"INSP"),"0%"),"-")</f>
         <v/>
       </c>
       <c r="F42" s="128" t="n"/>
-      <c r="H42" s="104">
+      <c r="H42" s="116">
         <f>IFERROR("Completion: "&amp;TEXT(COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"AP",'ASF Tracker'!$E$4:$E$1004,"Closed")/COUNTIFS('ASF Tracker'!$B$4:$B$1004,"&lt;&gt;",'ASF Tracker'!$G$4:$G$1004,"AP"),"0%"),"-")</f>
         <v/>
       </c>
@@ -30308,8 +30333,8 @@
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E39:F39"/>
+    <mergeCell ref="A19:J19"/>
     <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A19:J19"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="H39:I39"/>
     <mergeCell ref="H25:I25"/>

</xml_diff>